<commit_message>
updates to supplementary tables
</commit_message>
<xml_diff>
--- a/figures/supplement/Supplementary_Tables.xlsx
+++ b/figures/supplement/Supplementary_Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/magu/Documents/repos/cnv-ukb/figures/supplement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B596252-2B12-B049-B4A2-239ABBC7AC29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07627A5B-1E23-6C47-986C-45B5FD3753C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="460" windowWidth="23900" windowHeight="12700" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="460" windowWidth="23900" windowHeight="12700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table-S2b" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="111">
-  <si>
-    <t>Pathway Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="142">
   <si>
     <t>Delta z</t>
   </si>
@@ -249,9 +246,6 @@
     <t>BRCA1-A complex</t>
   </si>
   <si>
-    <t>HPO Term</t>
-  </si>
-  <si>
     <t>Deletion z</t>
   </si>
   <si>
@@ -358,6 +352,105 @@
   </si>
   <si>
     <t>HPO ID</t>
+  </si>
+  <si>
+    <t>Duplication-intolerant GO Name</t>
+  </si>
+  <si>
+    <t>Deletion-intolerant GO Pathway</t>
+  </si>
+  <si>
+    <t>Duplication-intolerant HPO Term</t>
+  </si>
+  <si>
+    <t>HP:0000707</t>
+  </si>
+  <si>
+    <t>Abnormality of the nervous system</t>
+  </si>
+  <si>
+    <t>HP:0012638</t>
+  </si>
+  <si>
+    <t>Abnormality of nervous system physiology</t>
+  </si>
+  <si>
+    <t>HP:0012759</t>
+  </si>
+  <si>
+    <t>Neurodevelopmental abnormality</t>
+  </si>
+  <si>
+    <t>HP:0000007</t>
+  </si>
+  <si>
+    <t>Autosomal recessive inheritance</t>
+  </si>
+  <si>
+    <t>HP:0012639</t>
+  </si>
+  <si>
+    <t>Abnormality of nervous system morphology</t>
+  </si>
+  <si>
+    <t>HP:0003011</t>
+  </si>
+  <si>
+    <t>Abnormality of the musculature</t>
+  </si>
+  <si>
+    <t>HP:0012373</t>
+  </si>
+  <si>
+    <t>Abnormal eye physiology</t>
+  </si>
+  <si>
+    <t>HP:0000478</t>
+  </si>
+  <si>
+    <t>Abnormality of the eye</t>
+  </si>
+  <si>
+    <t>HP:0100022</t>
+  </si>
+  <si>
+    <t>Abnormality of movement</t>
+  </si>
+  <si>
+    <t>HP:0012758</t>
+  </si>
+  <si>
+    <t>Neurodevelopmental delay</t>
+  </si>
+  <si>
+    <t>HP:0001249</t>
+  </si>
+  <si>
+    <t>Intellectual disability</t>
+  </si>
+  <si>
+    <t>HP:0012443</t>
+  </si>
+  <si>
+    <t>Abnormality of brain morphology</t>
+  </si>
+  <si>
+    <t>HP:0002011</t>
+  </si>
+  <si>
+    <t>Morphological abnormality of the central nervous system</t>
+  </si>
+  <si>
+    <t>HP:0011842</t>
+  </si>
+  <si>
+    <t>Abnormality of skeletal morphology</t>
+  </si>
+  <si>
+    <t>HP:0000924</t>
+  </si>
+  <si>
+    <t>Abnormality of the skeletal system</t>
   </si>
 </sst>
 </file>
@@ -420,7 +513,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -428,6 +521,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,27 +862,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="47.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3">
         <v>0.33271360534299999</v>
@@ -799,10 +897,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3">
         <v>0.189600158736</v>
@@ -813,10 +911,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="3">
         <v>4.9380936501900001E-2</v>
@@ -827,10 +925,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
         <v>0.13420865516399999</v>
@@ -841,10 +939,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3">
         <v>0.21549005876300001</v>
@@ -855,10 +953,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3">
         <v>0.16714978497399999</v>
@@ -869,10 +967,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" s="3">
         <v>0.36244806636100002</v>
@@ -883,10 +981,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3">
         <v>0.23507595634299999</v>
@@ -897,10 +995,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" s="3">
         <v>0.24442900326200001</v>
@@ -911,10 +1009,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="3">
         <v>0.28981473930700002</v>
@@ -925,10 +1023,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" s="3">
         <v>0.37548788601999999</v>
@@ -939,10 +1037,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="3">
         <v>0.23733183807700001</v>
@@ -953,10 +1051,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" s="3">
         <v>0.28290486570899998</v>
@@ -967,10 +1065,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" s="3">
         <v>0.245928727854</v>
@@ -981,10 +1079,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="3">
         <v>0.152404738805</v>
@@ -1002,27 +1100,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="3">
         <v>0.46925974374700002</v>
@@ -1033,10 +1135,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3">
         <v>0.63087442108500003</v>
@@ -1047,10 +1149,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" s="3">
         <v>0.57609288718600005</v>
@@ -1061,10 +1163,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="3">
         <v>0.34345538307700002</v>
@@ -1075,10 +1177,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" s="3">
         <v>0.57644695570899995</v>
@@ -1089,10 +1191,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" s="3">
         <v>0.290704697013</v>
@@ -1103,10 +1205,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C8" s="3">
         <v>0.41680183621299999</v>
@@ -1117,10 +1219,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="3">
         <v>0.41680183621299999</v>
@@ -1131,10 +1233,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" s="3">
         <v>0.48812123530700002</v>
@@ -1145,10 +1247,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="3">
         <v>0.241222113264</v>
@@ -1159,10 +1261,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="3">
         <v>0.47979496749700001</v>
@@ -1173,10 +1275,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="3">
         <v>0.26719934912499999</v>
@@ -1187,10 +1289,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="3">
         <v>0.44881676881400001</v>
@@ -1201,10 +1303,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="3">
         <v>0.44881676881400001</v>
@@ -1215,10 +1317,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C16" s="3">
         <v>0.44358254731000002</v>
@@ -1236,27 +1338,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.5" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="3">
         <v>0.228987867495</v>
@@ -1267,10 +1373,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="3">
         <v>0.351471528112</v>
@@ -1281,10 +1387,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="3">
         <v>5.457295107E-2</v>
@@ -1295,10 +1401,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="3">
         <v>0.31397038513100001</v>
@@ -1309,10 +1415,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="3">
         <v>0.42250724922999999</v>
@@ -1323,10 +1429,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C7" s="3">
         <v>0.37992189663100001</v>
@@ -1337,10 +1443,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
         <v>0.14732970318399999</v>
@@ -1351,10 +1457,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" s="3">
         <v>0.39743682348300002</v>
@@ -1365,10 +1471,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" s="3">
         <v>0.29339010670299998</v>
@@ -1379,10 +1485,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="3">
         <v>0.49221794131899999</v>
@@ -1393,10 +1499,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3">
         <v>0.23063132196300001</v>
@@ -1407,10 +1513,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="3">
         <v>0.37723737497100002</v>
@@ -1421,10 +1527,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C14" s="3">
         <v>0.30753289553199997</v>
@@ -1435,10 +1541,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C15" s="3">
         <v>0.34762906899599999</v>
@@ -1449,10 +1555,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C16" s="3">
         <v>0.69231658351500003</v>
@@ -1470,229 +1576,233 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0.46925974374700002</v>
+        <v>113</v>
+      </c>
+      <c r="C2">
+        <v>3.9648998352800002E-2</v>
       </c>
       <c r="D2" s="4">
-        <v>1.22091972601E-36</v>
+        <v>3.0951704671700001E-17</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>114</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" s="3">
-        <v>0.63087442108500003</v>
+        <v>115</v>
+      </c>
+      <c r="C3">
+        <v>3.9370588977500003E-2</v>
       </c>
       <c r="D3" s="4">
-        <v>2.91070317622E-32</v>
+        <v>1.9326108762100001E-16</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0.57609288718600005</v>
+        <v>117</v>
+      </c>
+      <c r="C4">
+        <v>3.7309550199099997E-2</v>
       </c>
       <c r="D4" s="4">
-        <v>9.3833946404700005E-32</v>
+        <v>5.0425492561099999E-15</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0.34345538307700002</v>
+        <v>119</v>
+      </c>
+      <c r="C5">
+        <v>3.9233483190499997E-2</v>
       </c>
       <c r="D5" s="4">
-        <v>2.5477105165000001E-30</v>
+        <v>2.07681277391E-14</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="3">
-        <v>0.57644695570899995</v>
+        <v>121</v>
+      </c>
+      <c r="C6">
+        <v>3.8851712588900002E-2</v>
       </c>
       <c r="D6" s="4">
-        <v>2.8335818274999998E-29</v>
+        <v>5.6674081974600001E-14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>122</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="3">
-        <v>0.290704697013</v>
+        <v>123</v>
+      </c>
+      <c r="C7">
+        <v>3.86214966341E-2</v>
       </c>
       <c r="D7" s="4">
-        <v>4.2880557396899997E-27</v>
+        <v>9.5842246262799997E-14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0.41680183621299999</v>
+        <v>125</v>
+      </c>
+      <c r="C8">
+        <v>3.73088368413E-2</v>
       </c>
       <c r="D8" s="4">
-        <v>6.4067325662900001E-26</v>
+        <v>9.8085587901399999E-14</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0.41680183621299999</v>
+        <v>127</v>
+      </c>
+      <c r="C9">
+        <v>3.9384266460100001E-2</v>
       </c>
       <c r="D9" s="4">
-        <v>6.4067325662900001E-26</v>
+        <v>1.1565044201599999E-13</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="3">
-        <v>0.48812123530700002</v>
+        <v>129</v>
+      </c>
+      <c r="C10">
+        <v>3.6173311961499997E-2</v>
       </c>
       <c r="D10" s="4">
-        <v>3.3779024128600003E-24</v>
+        <v>6.2655992045799999E-13</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>130</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="3">
-        <v>0.241222113264</v>
+        <v>131</v>
+      </c>
+      <c r="C11">
+        <v>3.6115818927100002E-2</v>
       </c>
       <c r="D11" s="4">
-        <v>1.7576078268900001E-23</v>
+        <v>8.8125186381900004E-13</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0.47979496749700001</v>
+        <v>133</v>
+      </c>
+      <c r="C12">
+        <v>3.5805482805699999E-2</v>
       </c>
       <c r="D12" s="4">
-        <v>2.43589457287E-23</v>
+        <v>1.02087547124E-12</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="3">
-        <v>0.26719934912499999</v>
+        <v>135</v>
+      </c>
+      <c r="C13">
+        <v>3.7980741057E-2</v>
       </c>
       <c r="D13" s="4">
-        <v>2.6925247226299999E-22</v>
+        <v>1.3182966569899999E-12</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>136</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0.44881676881400001</v>
+        <v>137</v>
+      </c>
+      <c r="C14">
+        <v>3.9044483991699998E-2</v>
       </c>
       <c r="D14" s="4">
-        <v>9.7972554049599999E-22</v>
+        <v>2.07751384459E-12</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
-      </c>
-      <c r="C15" s="3">
-        <v>0.44881676881400001</v>
+        <v>139</v>
+      </c>
+      <c r="C15">
+        <v>3.9994577546999997E-2</v>
       </c>
       <c r="D15" s="4">
-        <v>9.7972554049599999E-22</v>
+        <v>2.24180155827E-12</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0.44358254731000002</v>
+        <v>141</v>
+      </c>
+      <c r="C16">
+        <v>4.0533906437500003E-2</v>
       </c>
       <c r="D16" s="4">
-        <v>3.3219254187300001E-21</v>
+        <v>4.5560070042599999E-12</v>
       </c>
     </row>
   </sheetData>
@@ -1707,18 +1817,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="3">
         <v>2.8697339525899999</v>
@@ -1729,7 +1839,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" s="3">
         <v>2.1358837038499998</v>
@@ -1740,7 +1850,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4" s="3">
         <v>1.78994581112</v>
@@ -1751,7 +1861,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="3">
         <v>1.06269059195</v>
@@ -1762,7 +1872,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="3">
         <v>1.0477659827200001</v>
@@ -1773,7 +1883,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3">
         <v>1.03329043653</v>
@@ -1784,7 +1894,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="3">
         <v>0.90187806554000005</v>
@@ -1795,7 +1905,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="3">
         <v>0.85822897621100003</v>
@@ -1806,7 +1916,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10" s="3">
         <v>0.79987810087699995</v>
@@ -1817,7 +1927,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11" s="3">
         <v>0.79894454951899996</v>
@@ -1828,7 +1938,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B12" s="3">
         <v>0.79880526206900004</v>
@@ -1839,7 +1949,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B13" s="3">
         <v>0.79801540557299999</v>
@@ -1850,7 +1960,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B14" s="3">
         <v>0.79251390682</v>
@@ -1861,7 +1971,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B15" s="3">
         <v>0.792138469048</v>
@@ -1872,7 +1982,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B16" s="3">
         <v>0.78998870964000001</v>
@@ -1893,18 +2003,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="3">
         <v>0.56571583278299997</v>
@@ -1915,7 +2025,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B3" s="3">
         <v>0.56542216977199999</v>
@@ -1926,7 +2036,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B4" s="3">
         <v>0.56539541306700003</v>
@@ -1937,7 +2047,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B5" s="3">
         <v>0.56481054115100005</v>
@@ -1948,7 +2058,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B6" s="3">
         <v>0.56465142040600003</v>
@@ -1959,7 +2069,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B7" s="3">
         <v>0.56437396321599997</v>
@@ -1970,7 +2080,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B8" s="3">
         <v>0.56433688851999997</v>
@@ -1981,7 +2091,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B9" s="3">
         <v>0.56426679149199999</v>
@@ -1992,7 +2102,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B10" s="3">
         <v>0.56419427552300006</v>
@@ -2003,7 +2113,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>0.56419316264099995</v>
@@ -2014,7 +2124,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B12" s="3">
         <v>0.56409321011699998</v>
@@ -2025,7 +2135,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3">
         <v>0.56402182156199998</v>
@@ -2036,7 +2146,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B14" s="3">
         <v>0.56391999286700001</v>
@@ -2047,7 +2157,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B15" s="3">
         <v>0.56391999286700001</v>
@@ -2058,7 +2168,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B16" s="3">
         <v>0.56387102606299999</v>

</xml_diff>